<commit_message>
Craigdell: treat DOWN-tagged unit 004A as non-revenue
A unit whose AppFolio tag is DOWN is offline, not a rentable vacancy.
Normalize it to the Down status in intake so expand_nonrev nets it to
zero (rent = market, offsetting negative concession) and drops it out of
both the occupied and vacant buckets. Totals still tie to source
(97 units / 76,200 SF / 85,460 mkt / 79,227 rent). Occupancy now
89 occ / 7 vac / 1 non-revenue.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QgY3cyE49yD2oQoBHHNQL4
</commit_message>
<xml_diff>
--- a/examples/outputs/Birgo RR Exhibits - Craigdell Gardensv07.13.26.xlsx
+++ b/examples/outputs/Birgo RR Exhibits - Craigdell Gardensv07.13.26.xlsx
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="W50" s="27" t="n">
-        <v>0</v>
+        <v>-895</v>
       </c>
     </row>
     <row r="51">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="K13" s="36" t="inlineStr">
         <is>
-          <t>Vacant</t>
+          <t>Down</t>
         </is>
       </c>
       <c r="L13" s="55" t="n">
@@ -3270,17 +3270,17 @@
       </c>
       <c r="Q13" s="57" t="inlineStr">
         <is>
-          <t>Vac</t>
+          <t>Down</t>
         </is>
       </c>
       <c r="U13" s="58" t="n">
         <v>895</v>
       </c>
       <c r="V13" s="58" t="n">
-        <v>0</v>
+        <v>895</v>
       </c>
       <c r="W13" s="58" t="n">
-        <v>0</v>
+        <v>-895</v>
       </c>
       <c r="X13" s="58" t="n">
         <v>0</v>
@@ -9154,7 +9154,7 @@
         <v>79227</v>
       </c>
       <c r="W105" s="64" t="n">
-        <v>0</v>
+        <v>-895</v>
       </c>
       <c r="X105" s="64" t="n">
         <v>0</v>
@@ -9186,7 +9186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:AB128"/>
+  <dimension ref="A3:AD128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.6" customWidth="1" min="1" max="1"/>
@@ -9210,6 +9210,7 @@
     <col width="24" customWidth="1" min="22" max="22"/>
     <col width="12.1" customWidth="1" min="25" max="25"/>
     <col width="13" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="3">
@@ -9718,6 +9719,11 @@
           <t>Other Income</t>
         </is>
       </c>
+      <c r="AD30" s="67" t="inlineStr">
+        <is>
+          <t>Concessions</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="67" t="inlineStr">
@@ -9838,6 +9844,11 @@
       <c r="AB31" s="67" t="inlineStr">
         <is>
           <t>Monthly Charges</t>
+        </is>
+      </c>
+      <c r="AD31" s="67" t="inlineStr">
+        <is>
+          <t>Concession</t>
         </is>
       </c>
     </row>
@@ -9907,8 +9918,9 @@
         <f>SUM(AB32:AB32)</f>
         <v/>
       </c>
-      <c r="S32" s="81" t="n">
-        <v>0</v>
+      <c r="S32" s="81">
+        <f>AD32</f>
+        <v/>
       </c>
       <c r="T32" s="81" t="n">
         <v>0</v>
@@ -9984,8 +9996,9 @@
         <f>SUM(AB33:AB33)</f>
         <v/>
       </c>
-      <c r="S33" s="81" t="n">
-        <v>0</v>
+      <c r="S33" s="81">
+        <f>AD33</f>
+        <v/>
       </c>
       <c r="T33" s="81" t="n">
         <v>0</v>
@@ -10061,8 +10074,9 @@
         <f>SUM(AB34:AB34)</f>
         <v/>
       </c>
-      <c r="S34" s="81" t="n">
-        <v>0</v>
+      <c r="S34" s="81">
+        <f>AD34</f>
+        <v/>
       </c>
       <c r="T34" s="81" t="n">
         <v>0</v>
@@ -10138,8 +10152,9 @@
         <f>SUM(AB35:AB35)</f>
         <v/>
       </c>
-      <c r="S35" s="81" t="n">
-        <v>0</v>
+      <c r="S35" s="81">
+        <f>AD35</f>
+        <v/>
       </c>
       <c r="T35" s="81" t="n">
         <v>0</v>
@@ -10218,8 +10233,9 @@
         <f>SUM(AB36:AB36)</f>
         <v/>
       </c>
-      <c r="S36" s="81" t="n">
-        <v>0</v>
+      <c r="S36" s="81">
+        <f>AD36</f>
+        <v/>
       </c>
       <c r="T36" s="81" t="n">
         <v>0</v>
@@ -10229,83 +10245,76 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="83">
+      <c r="A37" s="72">
         <f>$D$21</f>
         <v/>
       </c>
-      <c r="B37" s="83">
+      <c r="B37" s="72">
         <f>B36+1</f>
         <v/>
       </c>
-      <c r="C37" s="83">
+      <c r="C37" s="72">
         <f>IF(K37="Vacant","Vac",IF(K37="Model","Model",IF(K37="Admin","Admin",IF(K37="Down","Down",IF(K37="Super","Super","Occ")))))</f>
         <v/>
       </c>
-      <c r="D37" s="83">
+      <c r="D37" s="72">
         <f>INDEX($C$5:$C$8,MATCH(I37,$D$5:$D$8,0))</f>
         <v/>
       </c>
-      <c r="E37" s="83">
+      <c r="E37" s="72">
         <f>INDEX($E$5:$E$8,MATCH(D37,$C$5:$C$8,0))</f>
         <v/>
       </c>
-      <c r="F37" s="83">
+      <c r="F37" s="72">
         <f>INDEX($F$5:$F$8,MATCH(D37,$C$5:$C$8,0))</f>
         <v/>
       </c>
-      <c r="G37" s="83">
+      <c r="G37" s="72">
         <f>INDEX($G$5:$G$8,MATCH(D37,$C$5:$C$8,0))</f>
         <v/>
       </c>
-      <c r="H37" s="83" t="inlineStr">
+      <c r="H37" s="72" t="inlineStr">
         <is>
           <t>004A</t>
         </is>
       </c>
-      <c r="I37" s="83" t="inlineStr">
+      <c r="I37" s="72" t="inlineStr">
         <is>
           <t>2/1</t>
         </is>
       </c>
-      <c r="J37" s="84" t="n">
+      <c r="J37" s="80" t="n">
         <v>850</v>
       </c>
-      <c r="K37" s="83" t="inlineStr">
-        <is>
-          <t>Vacant</t>
-        </is>
-      </c>
-      <c r="L37" s="85" t="n">
+      <c r="K37" s="72" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="L37" s="81" t="n">
         <v>895</v>
       </c>
-      <c r="M37" s="85">
+      <c r="M37" s="81">
         <f>Y37</f>
         <v/>
       </c>
-      <c r="N37" s="86" t="n"/>
-      <c r="O37" s="86" t="n"/>
-      <c r="P37" s="86" t="n"/>
-      <c r="Q37" s="86" t="n"/>
-      <c r="R37" s="85">
+      <c r="R37" s="81">
         <f>SUM(AB37:AB37)</f>
         <v/>
       </c>
-      <c r="S37" s="85" t="n">
-        <v>0</v>
-      </c>
-      <c r="T37" s="85" t="n">
-        <v>0</v>
-      </c>
-      <c r="U37" s="86" t="n"/>
-      <c r="V37" s="86" t="n"/>
-      <c r="W37" s="86" t="n"/>
-      <c r="X37" s="86" t="n"/>
-      <c r="Y37" s="85" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z37" s="86" t="n"/>
-      <c r="AA37" s="86" t="n"/>
-      <c r="AB37" s="86" t="n"/>
+      <c r="S37" s="81">
+        <f>AD37</f>
+        <v/>
+      </c>
+      <c r="T37" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y37" s="81" t="n">
+        <v>895</v>
+      </c>
+      <c r="AD37" s="81" t="n">
+        <v>-895</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="72">
@@ -10374,8 +10383,9 @@
         <f>SUM(AB38:AB38)</f>
         <v/>
       </c>
-      <c r="S38" s="81" t="n">
-        <v>0</v>
+      <c r="S38" s="81">
+        <f>AD38</f>
+        <v/>
       </c>
       <c r="T38" s="81" t="n">
         <v>0</v>
@@ -10451,8 +10461,9 @@
         <f>SUM(AB39:AB39)</f>
         <v/>
       </c>
-      <c r="S39" s="81" t="n">
-        <v>0</v>
+      <c r="S39" s="81">
+        <f>AD39</f>
+        <v/>
       </c>
       <c r="T39" s="81" t="n">
         <v>0</v>
@@ -10528,8 +10539,9 @@
         <f>SUM(AB40:AB40)</f>
         <v/>
       </c>
-      <c r="S40" s="81" t="n">
-        <v>0</v>
+      <c r="S40" s="81">
+        <f>AD40</f>
+        <v/>
       </c>
       <c r="T40" s="81" t="n">
         <v>0</v>
@@ -10605,8 +10617,9 @@
         <f>SUM(AB41:AB41)</f>
         <v/>
       </c>
-      <c r="S41" s="81" t="n">
-        <v>0</v>
+      <c r="S41" s="81">
+        <f>AD41</f>
+        <v/>
       </c>
       <c r="T41" s="81" t="n">
         <v>0</v>
@@ -10682,8 +10695,9 @@
         <f>SUM(AB42:AB42)</f>
         <v/>
       </c>
-      <c r="S42" s="81" t="n">
-        <v>0</v>
+      <c r="S42" s="81">
+        <f>AD42</f>
+        <v/>
       </c>
       <c r="T42" s="81" t="n">
         <v>0</v>
@@ -10759,8 +10773,9 @@
         <f>SUM(AB43:AB43)</f>
         <v/>
       </c>
-      <c r="S43" s="81" t="n">
-        <v>0</v>
+      <c r="S43" s="81">
+        <f>AD43</f>
+        <v/>
       </c>
       <c r="T43" s="81" t="n">
         <v>0</v>
@@ -10839,8 +10854,9 @@
         <f>SUM(AB44:AB44)</f>
         <v/>
       </c>
-      <c r="S44" s="81" t="n">
-        <v>0</v>
+      <c r="S44" s="81">
+        <f>AD44</f>
+        <v/>
       </c>
       <c r="T44" s="81" t="n">
         <v>0</v>
@@ -10911,8 +10927,9 @@
         <f>SUM(AB45:AB45)</f>
         <v/>
       </c>
-      <c r="S45" s="85" t="n">
-        <v>0</v>
+      <c r="S45" s="85">
+        <f>AD45</f>
+        <v/>
       </c>
       <c r="T45" s="85" t="n">
         <v>0</v>
@@ -10927,6 +10944,8 @@
       <c r="Z45" s="86" t="n"/>
       <c r="AA45" s="86" t="n"/>
       <c r="AB45" s="86" t="n"/>
+      <c r="AC45" s="86" t="n"/>
+      <c r="AD45" s="86" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="72">
@@ -10995,8 +11014,9 @@
         <f>SUM(AB46:AB46)</f>
         <v/>
       </c>
-      <c r="S46" s="81" t="n">
-        <v>0</v>
+      <c r="S46" s="81">
+        <f>AD46</f>
+        <v/>
       </c>
       <c r="T46" s="81" t="n">
         <v>0</v>
@@ -11075,8 +11095,9 @@
         <f>SUM(AB47:AB47)</f>
         <v/>
       </c>
-      <c r="S47" s="81" t="n">
-        <v>0</v>
+      <c r="S47" s="81">
+        <f>AD47</f>
+        <v/>
       </c>
       <c r="T47" s="81" t="n">
         <v>0</v>
@@ -11149,8 +11170,9 @@
         <f>SUM(AB48:AB48)</f>
         <v/>
       </c>
-      <c r="S48" s="81" t="n">
-        <v>0</v>
+      <c r="S48" s="81">
+        <f>AD48</f>
+        <v/>
       </c>
       <c r="T48" s="81" t="n">
         <v>0</v>
@@ -11229,8 +11251,9 @@
         <f>SUM(AB49:AB49)</f>
         <v/>
       </c>
-      <c r="S49" s="81" t="n">
-        <v>0</v>
+      <c r="S49" s="81">
+        <f>AD49</f>
+        <v/>
       </c>
       <c r="T49" s="81" t="n">
         <v>0</v>
@@ -11306,8 +11329,9 @@
         <f>SUM(AB50:AB50)</f>
         <v/>
       </c>
-      <c r="S50" s="81" t="n">
-        <v>0</v>
+      <c r="S50" s="81">
+        <f>AD50</f>
+        <v/>
       </c>
       <c r="T50" s="81" t="n">
         <v>0</v>
@@ -11383,8 +11407,9 @@
         <f>SUM(AB51:AB51)</f>
         <v/>
       </c>
-      <c r="S51" s="81" t="n">
-        <v>0</v>
+      <c r="S51" s="81">
+        <f>AD51</f>
+        <v/>
       </c>
       <c r="T51" s="81" t="n">
         <v>0</v>
@@ -11455,8 +11480,9 @@
         <f>SUM(AB52:AB52)</f>
         <v/>
       </c>
-      <c r="S52" s="85" t="n">
-        <v>0</v>
+      <c r="S52" s="85">
+        <f>AD52</f>
+        <v/>
       </c>
       <c r="T52" s="85" t="n">
         <v>0</v>
@@ -11471,6 +11497,8 @@
       <c r="Z52" s="86" t="n"/>
       <c r="AA52" s="86" t="n"/>
       <c r="AB52" s="86" t="n"/>
+      <c r="AC52" s="86" t="n"/>
+      <c r="AD52" s="86" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="72">
@@ -11539,8 +11567,9 @@
         <f>SUM(AB53:AB53)</f>
         <v/>
       </c>
-      <c r="S53" s="81" t="n">
-        <v>0</v>
+      <c r="S53" s="81">
+        <f>AD53</f>
+        <v/>
       </c>
       <c r="T53" s="81" t="n">
         <v>0</v>
@@ -11611,8 +11640,9 @@
         <f>SUM(AB54:AB54)</f>
         <v/>
       </c>
-      <c r="S54" s="85" t="n">
-        <v>0</v>
+      <c r="S54" s="85">
+        <f>AD54</f>
+        <v/>
       </c>
       <c r="T54" s="85" t="n">
         <v>0</v>
@@ -11627,6 +11657,8 @@
       <c r="Z54" s="86" t="n"/>
       <c r="AA54" s="86" t="n"/>
       <c r="AB54" s="86" t="n"/>
+      <c r="AC54" s="86" t="n"/>
+      <c r="AD54" s="86" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="72">
@@ -11692,8 +11724,9 @@
         <f>SUM(AB55:AB55)</f>
         <v/>
       </c>
-      <c r="S55" s="81" t="n">
-        <v>0</v>
+      <c r="S55" s="81">
+        <f>AD55</f>
+        <v/>
       </c>
       <c r="T55" s="81" t="n">
         <v>0</v>
@@ -11769,8 +11802,9 @@
         <f>SUM(AB56:AB56)</f>
         <v/>
       </c>
-      <c r="S56" s="81" t="n">
-        <v>0</v>
+      <c r="S56" s="81">
+        <f>AD56</f>
+        <v/>
       </c>
       <c r="T56" s="81" t="n">
         <v>0</v>
@@ -11846,8 +11880,9 @@
         <f>SUM(AB57:AB57)</f>
         <v/>
       </c>
-      <c r="S57" s="81" t="n">
-        <v>0</v>
+      <c r="S57" s="81">
+        <f>AD57</f>
+        <v/>
       </c>
       <c r="T57" s="81" t="n">
         <v>0</v>
@@ -11923,8 +11958,9 @@
         <f>SUM(AB58:AB58)</f>
         <v/>
       </c>
-      <c r="S58" s="81" t="n">
-        <v>0</v>
+      <c r="S58" s="81">
+        <f>AD58</f>
+        <v/>
       </c>
       <c r="T58" s="81" t="n">
         <v>0</v>
@@ -12000,8 +12036,9 @@
         <f>SUM(AB59:AB59)</f>
         <v/>
       </c>
-      <c r="S59" s="81" t="n">
-        <v>0</v>
+      <c r="S59" s="81">
+        <f>AD59</f>
+        <v/>
       </c>
       <c r="T59" s="81" t="n">
         <v>0</v>
@@ -12077,8 +12114,9 @@
         <f>SUM(AB60:AB60)</f>
         <v/>
       </c>
-      <c r="S60" s="81" t="n">
-        <v>0</v>
+      <c r="S60" s="81">
+        <f>AD60</f>
+        <v/>
       </c>
       <c r="T60" s="81" t="n">
         <v>0</v>
@@ -12154,8 +12192,9 @@
         <f>SUM(AB61:AB61)</f>
         <v/>
       </c>
-      <c r="S61" s="81" t="n">
-        <v>0</v>
+      <c r="S61" s="81">
+        <f>AD61</f>
+        <v/>
       </c>
       <c r="T61" s="81" t="n">
         <v>0</v>
@@ -12231,8 +12270,9 @@
         <f>SUM(AB62:AB62)</f>
         <v/>
       </c>
-      <c r="S62" s="81" t="n">
-        <v>0</v>
+      <c r="S62" s="81">
+        <f>AD62</f>
+        <v/>
       </c>
       <c r="T62" s="81" t="n">
         <v>0</v>
@@ -12308,8 +12348,9 @@
         <f>SUM(AB63:AB63)</f>
         <v/>
       </c>
-      <c r="S63" s="81" t="n">
-        <v>0</v>
+      <c r="S63" s="81">
+        <f>AD63</f>
+        <v/>
       </c>
       <c r="T63" s="81" t="n">
         <v>0</v>
@@ -12385,8 +12426,9 @@
         <f>SUM(AB64:AB64)</f>
         <v/>
       </c>
-      <c r="S64" s="81" t="n">
-        <v>0</v>
+      <c r="S64" s="81">
+        <f>AD64</f>
+        <v/>
       </c>
       <c r="T64" s="81" t="n">
         <v>0</v>
@@ -12462,8 +12504,9 @@
         <f>SUM(AB65:AB65)</f>
         <v/>
       </c>
-      <c r="S65" s="81" t="n">
-        <v>0</v>
+      <c r="S65" s="81">
+        <f>AD65</f>
+        <v/>
       </c>
       <c r="T65" s="81" t="n">
         <v>0</v>
@@ -12534,8 +12577,9 @@
         <f>SUM(AB66:AB66)</f>
         <v/>
       </c>
-      <c r="S66" s="85" t="n">
-        <v>0</v>
+      <c r="S66" s="85">
+        <f>AD66</f>
+        <v/>
       </c>
       <c r="T66" s="85" t="n">
         <v>0</v>
@@ -12550,6 +12594,8 @@
       <c r="Z66" s="86" t="n"/>
       <c r="AA66" s="86" t="n"/>
       <c r="AB66" s="86" t="n"/>
+      <c r="AC66" s="86" t="n"/>
+      <c r="AD66" s="86" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="72">
@@ -12618,8 +12664,9 @@
         <f>SUM(AB67:AB67)</f>
         <v/>
       </c>
-      <c r="S67" s="81" t="n">
-        <v>0</v>
+      <c r="S67" s="81">
+        <f>AD67</f>
+        <v/>
       </c>
       <c r="T67" s="81" t="n">
         <v>0</v>
@@ -12698,8 +12745,9 @@
         <f>SUM(AB68:AB68)</f>
         <v/>
       </c>
-      <c r="S68" s="81" t="n">
-        <v>0</v>
+      <c r="S68" s="81">
+        <f>AD68</f>
+        <v/>
       </c>
       <c r="T68" s="81" t="n">
         <v>0</v>
@@ -12775,8 +12823,9 @@
         <f>SUM(AB69:AB69)</f>
         <v/>
       </c>
-      <c r="S69" s="81" t="n">
-        <v>0</v>
+      <c r="S69" s="81">
+        <f>AD69</f>
+        <v/>
       </c>
       <c r="T69" s="81" t="n">
         <v>0</v>
@@ -12852,8 +12901,9 @@
         <f>SUM(AB70:AB70)</f>
         <v/>
       </c>
-      <c r="S70" s="81" t="n">
-        <v>0</v>
+      <c r="S70" s="81">
+        <f>AD70</f>
+        <v/>
       </c>
       <c r="T70" s="81" t="n">
         <v>0</v>
@@ -12932,8 +12982,9 @@
         <f>SUM(AB71:AB71)</f>
         <v/>
       </c>
-      <c r="S71" s="81" t="n">
-        <v>0</v>
+      <c r="S71" s="81">
+        <f>AD71</f>
+        <v/>
       </c>
       <c r="T71" s="81" t="n">
         <v>0</v>
@@ -13009,8 +13060,9 @@
         <f>SUM(AB72:AB72)</f>
         <v/>
       </c>
-      <c r="S72" s="81" t="n">
-        <v>0</v>
+      <c r="S72" s="81">
+        <f>AD72</f>
+        <v/>
       </c>
       <c r="T72" s="81" t="n">
         <v>0</v>
@@ -13086,8 +13138,9 @@
         <f>SUM(AB73:AB73)</f>
         <v/>
       </c>
-      <c r="S73" s="81" t="n">
-        <v>0</v>
+      <c r="S73" s="81">
+        <f>AD73</f>
+        <v/>
       </c>
       <c r="T73" s="81" t="n">
         <v>0</v>
@@ -13163,8 +13216,9 @@
         <f>SUM(AB74:AB74)</f>
         <v/>
       </c>
-      <c r="S74" s="81" t="n">
-        <v>0</v>
+      <c r="S74" s="81">
+        <f>AD74</f>
+        <v/>
       </c>
       <c r="T74" s="81" t="n">
         <v>0</v>
@@ -13240,8 +13294,9 @@
         <f>SUM(AB75:AB75)</f>
         <v/>
       </c>
-      <c r="S75" s="81" t="n">
-        <v>0</v>
+      <c r="S75" s="81">
+        <f>AD75</f>
+        <v/>
       </c>
       <c r="T75" s="81" t="n">
         <v>0</v>
@@ -13320,8 +13375,9 @@
         <f>SUM(AB76:AB76)</f>
         <v/>
       </c>
-      <c r="S76" s="81" t="n">
-        <v>0</v>
+      <c r="S76" s="81">
+        <f>AD76</f>
+        <v/>
       </c>
       <c r="T76" s="81" t="n">
         <v>0</v>
@@ -13400,8 +13456,9 @@
         <f>SUM(AB77:AB77)</f>
         <v/>
       </c>
-      <c r="S77" s="81" t="n">
-        <v>0</v>
+      <c r="S77" s="81">
+        <f>AD77</f>
+        <v/>
       </c>
       <c r="T77" s="81" t="n">
         <v>0</v>
@@ -13480,8 +13537,9 @@
         <f>SUM(AB78:AB78)</f>
         <v/>
       </c>
-      <c r="S78" s="81" t="n">
-        <v>0</v>
+      <c r="S78" s="81">
+        <f>AD78</f>
+        <v/>
       </c>
       <c r="T78" s="81" t="n">
         <v>0</v>
@@ -13557,8 +13615,9 @@
         <f>SUM(AB79:AB79)</f>
         <v/>
       </c>
-      <c r="S79" s="81" t="n">
-        <v>0</v>
+      <c r="S79" s="81">
+        <f>AD79</f>
+        <v/>
       </c>
       <c r="T79" s="81" t="n">
         <v>0</v>
@@ -13634,8 +13693,9 @@
         <f>SUM(AB80:AB80)</f>
         <v/>
       </c>
-      <c r="S80" s="81" t="n">
-        <v>0</v>
+      <c r="S80" s="81">
+        <f>AD80</f>
+        <v/>
       </c>
       <c r="T80" s="81" t="n">
         <v>0</v>
@@ -13708,8 +13768,9 @@
         <f>SUM(AB81:AB81)</f>
         <v/>
       </c>
-      <c r="S81" s="81" t="n">
-        <v>0</v>
+      <c r="S81" s="81">
+        <f>AD81</f>
+        <v/>
       </c>
       <c r="T81" s="81" t="n">
         <v>0</v>
@@ -13788,8 +13849,9 @@
         <f>SUM(AB82:AB82)</f>
         <v/>
       </c>
-      <c r="S82" s="81" t="n">
-        <v>0</v>
+      <c r="S82" s="81">
+        <f>AD82</f>
+        <v/>
       </c>
       <c r="T82" s="81" t="n">
         <v>0</v>
@@ -13865,8 +13927,9 @@
         <f>SUM(AB83:AB83)</f>
         <v/>
       </c>
-      <c r="S83" s="81" t="n">
-        <v>0</v>
+      <c r="S83" s="81">
+        <f>AD83</f>
+        <v/>
       </c>
       <c r="T83" s="81" t="n">
         <v>0</v>
@@ -13942,8 +14005,9 @@
         <f>SUM(AB84:AB84)</f>
         <v/>
       </c>
-      <c r="S84" s="81" t="n">
-        <v>0</v>
+      <c r="S84" s="81">
+        <f>AD84</f>
+        <v/>
       </c>
       <c r="T84" s="81" t="n">
         <v>0</v>
@@ -14019,8 +14083,9 @@
         <f>SUM(AB85:AB85)</f>
         <v/>
       </c>
-      <c r="S85" s="81" t="n">
-        <v>0</v>
+      <c r="S85" s="81">
+        <f>AD85</f>
+        <v/>
       </c>
       <c r="T85" s="81" t="n">
         <v>0</v>
@@ -14096,8 +14161,9 @@
         <f>SUM(AB86:AB86)</f>
         <v/>
       </c>
-      <c r="S86" s="81" t="n">
-        <v>0</v>
+      <c r="S86" s="81">
+        <f>AD86</f>
+        <v/>
       </c>
       <c r="T86" s="81" t="n">
         <v>0</v>
@@ -14173,8 +14239,9 @@
         <f>SUM(AB87:AB87)</f>
         <v/>
       </c>
-      <c r="S87" s="81" t="n">
-        <v>0</v>
+      <c r="S87" s="81">
+        <f>AD87</f>
+        <v/>
       </c>
       <c r="T87" s="81" t="n">
         <v>0</v>
@@ -14250,8 +14317,9 @@
         <f>SUM(AB88:AB88)</f>
         <v/>
       </c>
-      <c r="S88" s="81" t="n">
-        <v>0</v>
+      <c r="S88" s="81">
+        <f>AD88</f>
+        <v/>
       </c>
       <c r="T88" s="81" t="n">
         <v>0</v>
@@ -14324,8 +14392,9 @@
         <f>SUM(AB89:AB89)</f>
         <v/>
       </c>
-      <c r="S89" s="81" t="n">
-        <v>0</v>
+      <c r="S89" s="81">
+        <f>AD89</f>
+        <v/>
       </c>
       <c r="T89" s="81" t="n">
         <v>0</v>
@@ -14401,8 +14470,9 @@
         <f>SUM(AB90:AB90)</f>
         <v/>
       </c>
-      <c r="S90" s="81" t="n">
-        <v>0</v>
+      <c r="S90" s="81">
+        <f>AD90</f>
+        <v/>
       </c>
       <c r="T90" s="81" t="n">
         <v>0</v>
@@ -14481,8 +14551,9 @@
         <f>SUM(AB91:AB91)</f>
         <v/>
       </c>
-      <c r="S91" s="81" t="n">
-        <v>0</v>
+      <c r="S91" s="81">
+        <f>AD91</f>
+        <v/>
       </c>
       <c r="T91" s="81" t="n">
         <v>0</v>
@@ -14558,8 +14629,9 @@
         <f>SUM(AB92:AB92)</f>
         <v/>
       </c>
-      <c r="S92" s="81" t="n">
-        <v>0</v>
+      <c r="S92" s="81">
+        <f>AD92</f>
+        <v/>
       </c>
       <c r="T92" s="81" t="n">
         <v>0</v>
@@ -14635,8 +14707,9 @@
         <f>SUM(AB93:AB93)</f>
         <v/>
       </c>
-      <c r="S93" s="81" t="n">
-        <v>0</v>
+      <c r="S93" s="81">
+        <f>AD93</f>
+        <v/>
       </c>
       <c r="T93" s="81" t="n">
         <v>0</v>
@@ -14715,8 +14788,9 @@
         <f>SUM(AB94:AB94)</f>
         <v/>
       </c>
-      <c r="S94" s="81" t="n">
-        <v>0</v>
+      <c r="S94" s="81">
+        <f>AD94</f>
+        <v/>
       </c>
       <c r="T94" s="81" t="n">
         <v>0</v>
@@ -14792,8 +14866,9 @@
         <f>SUM(AB95:AB95)</f>
         <v/>
       </c>
-      <c r="S95" s="81" t="n">
-        <v>0</v>
+      <c r="S95" s="81">
+        <f>AD95</f>
+        <v/>
       </c>
       <c r="T95" s="81" t="n">
         <v>0</v>
@@ -14869,8 +14944,9 @@
         <f>SUM(AB96:AB96)</f>
         <v/>
       </c>
-      <c r="S96" s="81" t="n">
-        <v>0</v>
+      <c r="S96" s="81">
+        <f>AD96</f>
+        <v/>
       </c>
       <c r="T96" s="81" t="n">
         <v>0</v>
@@ -14946,8 +15022,9 @@
         <f>SUM(AB97:AB97)</f>
         <v/>
       </c>
-      <c r="S97" s="81" t="n">
-        <v>0</v>
+      <c r="S97" s="81">
+        <f>AD97</f>
+        <v/>
       </c>
       <c r="T97" s="81" t="n">
         <v>0</v>
@@ -15020,8 +15097,9 @@
         <f>SUM(AB98:AB98)</f>
         <v/>
       </c>
-      <c r="S98" s="81" t="n">
-        <v>0</v>
+      <c r="S98" s="81">
+        <f>AD98</f>
+        <v/>
       </c>
       <c r="T98" s="81" t="n">
         <v>0</v>
@@ -15097,8 +15175,9 @@
         <f>SUM(AB99:AB99)</f>
         <v/>
       </c>
-      <c r="S99" s="81" t="n">
-        <v>0</v>
+      <c r="S99" s="81">
+        <f>AD99</f>
+        <v/>
       </c>
       <c r="T99" s="81" t="n">
         <v>0</v>
@@ -15177,8 +15256,9 @@
         <f>SUM(AB100:AB100)</f>
         <v/>
       </c>
-      <c r="S100" s="81" t="n">
-        <v>0</v>
+      <c r="S100" s="81">
+        <f>AD100</f>
+        <v/>
       </c>
       <c r="T100" s="81" t="n">
         <v>0</v>
@@ -15249,8 +15329,9 @@
         <f>SUM(AB101:AB101)</f>
         <v/>
       </c>
-      <c r="S101" s="85" t="n">
-        <v>0</v>
+      <c r="S101" s="85">
+        <f>AD101</f>
+        <v/>
       </c>
       <c r="T101" s="85" t="n">
         <v>0</v>
@@ -15265,6 +15346,8 @@
       <c r="Z101" s="86" t="n"/>
       <c r="AA101" s="86" t="n"/>
       <c r="AB101" s="86" t="n"/>
+      <c r="AC101" s="86" t="n"/>
+      <c r="AD101" s="86" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="72">
@@ -15333,8 +15416,9 @@
         <f>SUM(AB102:AB102)</f>
         <v/>
       </c>
-      <c r="S102" s="81" t="n">
-        <v>0</v>
+      <c r="S102" s="81">
+        <f>AD102</f>
+        <v/>
       </c>
       <c r="T102" s="81" t="n">
         <v>0</v>
@@ -15405,8 +15489,9 @@
         <f>SUM(AB103:AB103)</f>
         <v/>
       </c>
-      <c r="S103" s="85" t="n">
-        <v>0</v>
+      <c r="S103" s="85">
+        <f>AD103</f>
+        <v/>
       </c>
       <c r="T103" s="85" t="n">
         <v>0</v>
@@ -15421,6 +15506,8 @@
       <c r="Z103" s="86" t="n"/>
       <c r="AA103" s="86" t="n"/>
       <c r="AB103" s="86" t="n"/>
+      <c r="AC103" s="86" t="n"/>
+      <c r="AD103" s="86" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="72">
@@ -15489,8 +15576,9 @@
         <f>SUM(AB104:AB104)</f>
         <v/>
       </c>
-      <c r="S104" s="81" t="n">
-        <v>0</v>
+      <c r="S104" s="81">
+        <f>AD104</f>
+        <v/>
       </c>
       <c r="T104" s="81" t="n">
         <v>0</v>
@@ -15569,8 +15657,9 @@
         <f>SUM(AB105:AB105)</f>
         <v/>
       </c>
-      <c r="S105" s="81" t="n">
-        <v>0</v>
+      <c r="S105" s="81">
+        <f>AD105</f>
+        <v/>
       </c>
       <c r="T105" s="81" t="n">
         <v>0</v>
@@ -15646,8 +15735,9 @@
         <f>SUM(AB106:AB106)</f>
         <v/>
       </c>
-      <c r="S106" s="81" t="n">
-        <v>0</v>
+      <c r="S106" s="81">
+        <f>AD106</f>
+        <v/>
       </c>
       <c r="T106" s="81" t="n">
         <v>0</v>
@@ -15723,8 +15813,9 @@
         <f>SUM(AB107:AB107)</f>
         <v/>
       </c>
-      <c r="S107" s="81" t="n">
-        <v>0</v>
+      <c r="S107" s="81">
+        <f>AD107</f>
+        <v/>
       </c>
       <c r="T107" s="81" t="n">
         <v>0</v>
@@ -15803,8 +15894,9 @@
         <f>SUM(AB108:AB108)</f>
         <v/>
       </c>
-      <c r="S108" s="81" t="n">
-        <v>0</v>
+      <c r="S108" s="81">
+        <f>AD108</f>
+        <v/>
       </c>
       <c r="T108" s="81" t="n">
         <v>0</v>
@@ -15880,8 +15972,9 @@
         <f>SUM(AB109:AB109)</f>
         <v/>
       </c>
-      <c r="S109" s="81" t="n">
-        <v>0</v>
+      <c r="S109" s="81">
+        <f>AD109</f>
+        <v/>
       </c>
       <c r="T109" s="81" t="n">
         <v>0</v>
@@ -15957,8 +16050,9 @@
         <f>SUM(AB110:AB110)</f>
         <v/>
       </c>
-      <c r="S110" s="81" t="n">
-        <v>0</v>
+      <c r="S110" s="81">
+        <f>AD110</f>
+        <v/>
       </c>
       <c r="T110" s="81" t="n">
         <v>0</v>
@@ -16034,8 +16128,9 @@
         <f>SUM(AB111:AB111)</f>
         <v/>
       </c>
-      <c r="S111" s="81" t="n">
-        <v>0</v>
+      <c r="S111" s="81">
+        <f>AD111</f>
+        <v/>
       </c>
       <c r="T111" s="81" t="n">
         <v>0</v>
@@ -16111,8 +16206,9 @@
         <f>SUM(AB112:AB112)</f>
         <v/>
       </c>
-      <c r="S112" s="81" t="n">
-        <v>0</v>
+      <c r="S112" s="81">
+        <f>AD112</f>
+        <v/>
       </c>
       <c r="T112" s="81" t="n">
         <v>0</v>
@@ -16188,8 +16284,9 @@
         <f>SUM(AB113:AB113)</f>
         <v/>
       </c>
-      <c r="S113" s="81" t="n">
-        <v>0</v>
+      <c r="S113" s="81">
+        <f>AD113</f>
+        <v/>
       </c>
       <c r="T113" s="81" t="n">
         <v>0</v>
@@ -16265,8 +16362,9 @@
         <f>SUM(AB114:AB114)</f>
         <v/>
       </c>
-      <c r="S114" s="81" t="n">
-        <v>0</v>
+      <c r="S114" s="81">
+        <f>AD114</f>
+        <v/>
       </c>
       <c r="T114" s="81" t="n">
         <v>0</v>
@@ -16342,8 +16440,9 @@
         <f>SUM(AB115:AB115)</f>
         <v/>
       </c>
-      <c r="S115" s="81" t="n">
-        <v>0</v>
+      <c r="S115" s="81">
+        <f>AD115</f>
+        <v/>
       </c>
       <c r="T115" s="81" t="n">
         <v>0</v>
@@ -16419,8 +16518,9 @@
         <f>SUM(AB116:AB116)</f>
         <v/>
       </c>
-      <c r="S116" s="81" t="n">
-        <v>0</v>
+      <c r="S116" s="81">
+        <f>AD116</f>
+        <v/>
       </c>
       <c r="T116" s="81" t="n">
         <v>0</v>
@@ -16499,8 +16599,9 @@
         <f>SUM(AB117:AB117)</f>
         <v/>
       </c>
-      <c r="S117" s="81" t="n">
-        <v>0</v>
+      <c r="S117" s="81">
+        <f>AD117</f>
+        <v/>
       </c>
       <c r="T117" s="81" t="n">
         <v>0</v>
@@ -16576,8 +16677,9 @@
         <f>SUM(AB118:AB118)</f>
         <v/>
       </c>
-      <c r="S118" s="81" t="n">
-        <v>0</v>
+      <c r="S118" s="81">
+        <f>AD118</f>
+        <v/>
       </c>
       <c r="T118" s="81" t="n">
         <v>0</v>
@@ -16653,8 +16755,9 @@
         <f>SUM(AB119:AB119)</f>
         <v/>
       </c>
-      <c r="S119" s="81" t="n">
-        <v>0</v>
+      <c r="S119" s="81">
+        <f>AD119</f>
+        <v/>
       </c>
       <c r="T119" s="81" t="n">
         <v>0</v>
@@ -16730,8 +16833,9 @@
         <f>SUM(AB120:AB120)</f>
         <v/>
       </c>
-      <c r="S120" s="81" t="n">
-        <v>0</v>
+      <c r="S120" s="81">
+        <f>AD120</f>
+        <v/>
       </c>
       <c r="T120" s="81" t="n">
         <v>0</v>
@@ -16807,8 +16911,9 @@
         <f>SUM(AB121:AB121)</f>
         <v/>
       </c>
-      <c r="S121" s="81" t="n">
-        <v>0</v>
+      <c r="S121" s="81">
+        <f>AD121</f>
+        <v/>
       </c>
       <c r="T121" s="81" t="n">
         <v>0</v>
@@ -16884,8 +16989,9 @@
         <f>SUM(AB122:AB122)</f>
         <v/>
       </c>
-      <c r="S122" s="81" t="n">
-        <v>0</v>
+      <c r="S122" s="81">
+        <f>AD122</f>
+        <v/>
       </c>
       <c r="T122" s="81" t="n">
         <v>0</v>
@@ -16961,8 +17067,9 @@
         <f>SUM(AB123:AB123)</f>
         <v/>
       </c>
-      <c r="S123" s="81" t="n">
-        <v>0</v>
+      <c r="S123" s="81">
+        <f>AD123</f>
+        <v/>
       </c>
       <c r="T123" s="81" t="n">
         <v>0</v>
@@ -17041,8 +17148,9 @@
         <f>SUM(AB124:AB124)</f>
         <v/>
       </c>
-      <c r="S124" s="81" t="n">
-        <v>0</v>
+      <c r="S124" s="81">
+        <f>AD124</f>
+        <v/>
       </c>
       <c r="T124" s="81" t="n">
         <v>0</v>
@@ -17118,8 +17226,9 @@
         <f>SUM(AB125:AB125)</f>
         <v/>
       </c>
-      <c r="S125" s="81" t="n">
-        <v>0</v>
+      <c r="S125" s="81">
+        <f>AD125</f>
+        <v/>
       </c>
       <c r="T125" s="81" t="n">
         <v>0</v>
@@ -17195,8 +17304,9 @@
         <f>SUM(AB126:AB126)</f>
         <v/>
       </c>
-      <c r="S126" s="81" t="n">
-        <v>0</v>
+      <c r="S126" s="81">
+        <f>AD126</f>
+        <v/>
       </c>
       <c r="T126" s="81" t="n">
         <v>0</v>
@@ -17270,8 +17380,9 @@
         <f>SUM(AB127:AB127)</f>
         <v/>
       </c>
-      <c r="S127" s="85" t="n">
-        <v>0</v>
+      <c r="S127" s="85">
+        <f>AD127</f>
+        <v/>
       </c>
       <c r="T127" s="85" t="n">
         <v>0</v>
@@ -17286,6 +17397,8 @@
       <c r="Z127" s="86" t="n"/>
       <c r="AA127" s="86" t="n"/>
       <c r="AB127" s="86" t="n"/>
+      <c r="AC127" s="86" t="n"/>
+      <c r="AD127" s="86" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="72">
@@ -17354,8 +17467,9 @@
         <f>SUM(AB128:AB128)</f>
         <v/>
       </c>
-      <c r="S128" s="81" t="n">
-        <v>0</v>
+      <c r="S128" s="81">
+        <f>AD128</f>
+        <v/>
       </c>
       <c r="T128" s="81" t="n">
         <v>0</v>

</xml_diff>